<commit_message>
Fix Budget, Fees & Grades tabs — content was starting in the 2px margin column
These three tabs use a leading margin column (A width 2) with content meant to
start in column B, but the table code wrote the first column into A — crushing it
and shifting every column out of alignment (jumbled / cut off in Sheets & Excel).

Shifted the tables to start at column B (start_col=2) so each column lands in its
intended width, and repointed the named cells (BudgetPlanTotal/BudgetSpent →
C14/D14, FeeAmtTotal/FeePaidTotal → D15/E15) and the dashboard Budget donut to the
new Actual/Category columns. All KPI values are unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YnPMpeJWKT9dx5HR1K2in
</commit_message>
<xml_diff>
--- a/products/back-to-school-family-command-center/Back_to_School_Command_Center.xlsx
+++ b/products/back-to-school-family-command-center/Back_to_School_Command_Center.xlsx
@@ -51,14 +51,14 @@
     <definedName name="SupCost">'Supplies'!$E$5:$E$64</definedName>
     <definedName name="ClothItem">'Clothing'!$B$5:$B$44</definedName>
     <definedName name="ClothReady">'Clothing'!$D$5:$D$44</definedName>
-    <definedName name="BudgetPlan">'Budget'!$B$5:$B$13</definedName>
-    <definedName name="BudgetActual">'Budget'!$C$5:$C$13</definedName>
-    <definedName name="BudgetPlanTotal">'Budget'!$B$14</definedName>
-    <definedName name="BudgetSpent">'Budget'!$C$14</definedName>
-    <definedName name="FeeAmt">'Fees'!$C$5:$C$14</definedName>
-    <definedName name="FeePaid">'Fees'!$D$5:$D$14</definedName>
-    <definedName name="FeeAmtTotal">'Fees'!$C$15</definedName>
-    <definedName name="FeePaidTotal">'Fees'!$D$15</definedName>
+    <definedName name="BudgetPlan">'Budget'!$C$5:$C$13</definedName>
+    <definedName name="BudgetActual">'Budget'!$D$5:$D$13</definedName>
+    <definedName name="BudgetPlanTotal">'Budget'!$C$14</definedName>
+    <definedName name="BudgetSpent">'Budget'!$D$14</definedName>
+    <definedName name="FeeAmt">'Fees'!$D$5:$D$14</definedName>
+    <definedName name="FeePaid">'Fees'!$E$5:$E$14</definedName>
+    <definedName name="FeeAmtTotal">'Fees'!$D$15</definedName>
+    <definedName name="FeePaidTotal">'Fees'!$E$15</definedName>
     <definedName name="DocName">'Documents'!$A$5:$A$34</definedName>
     <definedName name="DocDone">'Documents'!$B$5:$B$34</definedName>
     <definedName name="HealthRange">'Family Dashboard'!$C$13:$C$18</definedName>
@@ -620,7 +620,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Budget'!C4</f>
+              <f>'Budget'!D4</f>
             </strRef>
           </tx>
           <spPr>
@@ -630,12 +630,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Budget'!$A$5:$A$13</f>
+              <f>'Budget'!$B$5:$B$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Budget'!$C$5:$C$13</f>
+              <f>'Budget'!$D$5:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -1164,269 +1164,269 @@
       <c r="F3" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Child</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Fee</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Owed</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Mateo</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Registration</t>
         </is>
-      </c>
-      <c r="C5" s="35" t="n">
-        <v>75</v>
       </c>
       <c r="D5" s="35" t="n">
         <v>75</v>
       </c>
-      <c r="E5" s="43">
-        <f>C5-D5</f>
+      <c r="E5" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="F5" s="43">
+        <f>D5-E5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Mateo</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Athletics</t>
         </is>
-      </c>
-      <c r="C6" s="37" t="n">
-        <v>120</v>
       </c>
       <c r="D6" s="37" t="n">
         <v>120</v>
       </c>
-      <c r="E6" s="34">
-        <f>C6-D6</f>
+      <c r="E6" s="37" t="n">
+        <v>120</v>
+      </c>
+      <c r="F6" s="34">
+        <f>D6-E6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Sofia</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Registration</t>
         </is>
-      </c>
-      <c r="C7" s="35" t="n">
-        <v>75</v>
       </c>
       <c r="D7" s="35" t="n">
         <v>75</v>
       </c>
-      <c r="E7" s="43">
-        <f>C7-D7</f>
+      <c r="E7" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="F7" s="43">
+        <f>D7-E7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Sofia</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="D8" s="37" t="n">
         <v>90</v>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="E8" s="37" t="n">
         <v>45</v>
       </c>
-      <c r="E8" s="34">
-        <f>C8-D8</f>
+      <c r="F8" s="34">
+        <f>D8-E8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Liam</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Registration</t>
         </is>
-      </c>
-      <c r="C9" s="35" t="n">
-        <v>50</v>
       </c>
       <c r="D9" s="35" t="n">
         <v>50</v>
       </c>
-      <c r="E9" s="43">
-        <f>C9-D9</f>
+      <c r="E9" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" s="43">
+        <f>D9-E9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Ava</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>Registration</t>
         </is>
-      </c>
-      <c r="C10" s="37" t="n">
-        <v>50</v>
       </c>
       <c r="D10" s="37" t="n">
         <v>50</v>
       </c>
-      <c r="E10" s="34">
-        <f>C10-D10</f>
+      <c r="E10" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="F10" s="34">
+        <f>D10-E10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Noah</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Registration</t>
         </is>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="D11" s="35" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="35" t="n">
+      <c r="E11" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="43">
-        <f>C11-D11</f>
+      <c r="F11" s="43">
+        <f>D11-E11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Emma</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Preschool deposit</t>
         </is>
-      </c>
-      <c r="C12" s="37" t="n">
-        <v>150</v>
       </c>
       <c r="D12" s="37" t="n">
         <v>150</v>
       </c>
-      <c r="E12" s="34">
-        <f>C12-D12</f>
+      <c r="E12" s="37" t="n">
+        <v>150</v>
+      </c>
+      <c r="F12" s="34">
+        <f>D12-E12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>PTA</t>
         </is>
-      </c>
-      <c r="C13" s="35" t="n">
-        <v>40</v>
       </c>
       <c r="D13" s="35" t="n">
         <v>40</v>
       </c>
-      <c r="E13" s="43">
-        <f>C13-D13</f>
+      <c r="E13" s="35" t="n">
+        <v>40</v>
+      </c>
+      <c r="F13" s="43">
+        <f>D13-E13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>Yearbooks x3</t>
         </is>
-      </c>
-      <c r="C14" s="37" t="n">
-        <v>90</v>
       </c>
       <c r="D14" s="37" t="n">
         <v>90</v>
       </c>
-      <c r="E14" s="34">
-        <f>C14-D14</f>
+      <c r="E14" s="37" t="n">
+        <v>90</v>
+      </c>
+      <c r="F14" s="34">
+        <f>D14-E14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="39">
-        <f>SUM(C5:C14)</f>
-        <v/>
-      </c>
+      <c r="C15" s="9" t="n"/>
       <c r="D15" s="39">
         <f>SUM(D5:D14)</f>
         <v/>
       </c>
       <c r="E15" s="39">
         <f>SUM(E5:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="39">
+        <f>SUM(F5:F14)</f>
         <v/>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E14">
+  <conditionalFormatting sqref="F5:F14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -3971,152 +3971,152 @@
       <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Child</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Mateo</t>
         </is>
       </c>
-      <c r="B5" s="46" t="inlineStr">
+      <c r="C5" s="46" t="inlineStr">
         <is>
           <t>A-</t>
         </is>
       </c>
-      <c r="C5" s="46" t="inlineStr"/>
       <c r="D5" s="46" t="inlineStr"/>
       <c r="E5" s="46" t="inlineStr"/>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="F5" s="46" t="inlineStr"/>
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Sofia</t>
         </is>
       </c>
-      <c r="B6" s="47" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>B+</t>
         </is>
       </c>
-      <c r="C6" s="47" t="inlineStr"/>
       <c r="D6" s="47" t="inlineStr"/>
       <c r="E6" s="47" t="inlineStr"/>
-      <c r="F6" s="22" t="inlineStr">
+      <c r="F6" s="47" t="inlineStr"/>
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Liam</t>
         </is>
       </c>
-      <c r="B7" s="46" t="inlineStr">
+      <c r="C7" s="46" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C7" s="46" t="inlineStr"/>
       <c r="D7" s="46" t="inlineStr"/>
       <c r="E7" s="46" t="inlineStr"/>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F7" s="46" t="inlineStr"/>
+      <c r="G7" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Ava</t>
         </is>
       </c>
-      <c r="B8" s="47" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>S+</t>
         </is>
       </c>
-      <c r="C8" s="47" t="inlineStr"/>
       <c r="D8" s="47" t="inlineStr"/>
       <c r="E8" s="47" t="inlineStr"/>
-      <c r="F8" s="22" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr"/>
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Noah</t>
         </is>
       </c>
-      <c r="B9" s="46" t="inlineStr">
+      <c r="C9" s="46" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C9" s="46" t="inlineStr"/>
       <c r="D9" s="46" t="inlineStr"/>
       <c r="E9" s="46" t="inlineStr"/>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="F9" s="46" t="inlineStr"/>
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Emma</t>
         </is>
       </c>
-      <c r="B10" s="47" t="inlineStr">
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>😊</t>
         </is>
       </c>
-      <c r="C10" s="47" t="inlineStr"/>
       <c r="D10" s="47" t="inlineStr"/>
       <c r="E10" s="47" t="inlineStr"/>
-      <c r="F10" s="22" t="inlineStr">
+      <c r="F10" s="47" t="inlineStr"/>
+      <c r="G10" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -9796,189 +9796,185 @@
       <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>School Supplies</t>
         </is>
       </c>
-      <c r="B5" s="35" t="n">
+      <c r="C5" s="35" t="n">
         <v>320</v>
       </c>
-      <c r="C5" s="35" t="n">
+      <c r="D5" s="35" t="n">
         <v>300</v>
       </c>
-      <c r="D5" s="36">
-        <f>B5-C5</f>
+      <c r="E5" s="36">
+        <f>C5-D5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="C6" s="37" t="n">
         <v>480</v>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="D6" s="37" t="n">
         <v>415</v>
       </c>
-      <c r="D6" s="38">
-        <f>B6-C6</f>
+      <c r="E6" s="38">
+        <f>C6-D6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Shoes</t>
         </is>
       </c>
-      <c r="B7" s="35" t="n">
+      <c r="C7" s="35" t="n">
         <v>300</v>
       </c>
-      <c r="C7" s="35" t="n">
+      <c r="D7" s="35" t="n">
         <v>255</v>
       </c>
-      <c r="D7" s="36">
-        <f>B7-C7</f>
+      <c r="E7" s="36">
+        <f>C7-D7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Uniforms</t>
         </is>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="C8" s="37" t="n">
         <v>250</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="D8" s="37" t="n">
         <v>210</v>
       </c>
-      <c r="D8" s="38">
-        <f>B8-C8</f>
+      <c r="E8" s="38">
+        <f>C8-D8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Backpacks &amp; Lunchboxes</t>
         </is>
       </c>
-      <c r="B9" s="35" t="n">
+      <c r="C9" s="35" t="n">
         <v>180</v>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="D9" s="35" t="n">
         <v>165</v>
       </c>
-      <c r="D9" s="36">
-        <f>B9-C9</f>
+      <c r="E9" s="36">
+        <f>C9-D9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Devices &amp; Tech</t>
         </is>
       </c>
-      <c r="B10" s="37" t="n">
+      <c r="C10" s="37" t="n">
         <v>280</v>
       </c>
-      <c r="C10" s="37" t="n">
+      <c r="D10" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="38">
-        <f>B10-C10</f>
+      <c r="E10" s="38">
+        <f>C10-D10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>School Fees</t>
         </is>
       </c>
-      <c r="B11" s="35" t="n">
+      <c r="C11" s="35" t="n">
         <v>380</v>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="D11" s="35" t="n">
         <v>300</v>
       </c>
-      <c r="D11" s="36">
-        <f>B11-C11</f>
+      <c r="E11" s="36">
+        <f>C11-D11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Extracurriculars</t>
         </is>
       </c>
-      <c r="B12" s="37" t="n">
+      <c r="C12" s="37" t="n">
         <v>200</v>
       </c>
-      <c r="C12" s="37" t="n">
+      <c r="D12" s="37" t="n">
         <v>120</v>
       </c>
-      <c r="D12" s="38">
-        <f>B12-C12</f>
+      <c r="E12" s="38">
+        <f>C12-D12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Haircuts &amp; Misc</t>
         </is>
       </c>
-      <c r="B13" s="35" t="n">
+      <c r="C13" s="35" t="n">
         <v>110</v>
       </c>
-      <c r="C13" s="35" t="n">
+      <c r="D13" s="35" t="n">
         <v>85</v>
       </c>
-      <c r="D13" s="36">
-        <f>B13-C13</f>
+      <c r="E13" s="36">
+        <f>C13-D13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
-      </c>
-      <c r="B14" s="39">
-        <f>SUM(B5:B13)</f>
-        <v/>
       </c>
       <c r="C14" s="39">
         <f>SUM(C5:C13)</f>
@@ -9988,6 +9984,10 @@
         <f>SUM(D5:D13)</f>
         <v/>
       </c>
+      <c r="E14" s="39">
+        <f>SUM(E5:E13)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
@@ -10054,10 +10054,10 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B15:E15"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B15:D15"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:C13">
+  <conditionalFormatting sqref="D5:D13">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>

</xml_diff>